<commit_message>
Version del proyecto al dia 25/09/2026
</commit_message>
<xml_diff>
--- a/Archivos/CONFIGURACION/Formulas.xlsx
+++ b/Archivos/CONFIGURACION/Formulas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Procesos_Uipath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\CONFIGURACION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F7146CF-5C54-450B-B8AD-BB04E57337CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CCF3FBD-4999-4008-B5B8-81945F84516A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -111,7 +111,7 @@
     <t>=IF(OR(M_VALUE_DINAMIC_="SÍ", AND(X_VALUE_DINAMIC_&lt;&gt;"", X_VALUE_DINAMIC_&lt;=8), AND(Y_VALUE_DINAMIC_&lt;&gt;"", Y_VALUE_DINAMIC_&lt;=8), AND(Z_VALUE_DINAMIC_&lt;&gt;"", Z_VALUE_DINAMIC_&lt;=8), AND(Q_VALUE_DINAMIC_&lt;&gt;"", Q_VALUE_DINAMIC_&lt;=3), AND(AD_VALUE_DINAMIC_&lt;&gt;"", AD_VALUE_DINAMIC_&lt;=8), AND(AE4&lt;&gt;"", AE4&lt;=8),AND(N_VALUE_DINAMIC_&lt;&gt;"", N_VALUE_DINAMIC_&lt;=8)), "Alerta", "Correcto")</t>
   </si>
   <si>
-    <t>=CONCATENATE("?gid=",BC1,"#gid=",BC1,"&amp;range=A",ROW())</t>
+    <t>=CONCATENATE("?gid=",BB$1,"#gid=",$BB$1,"&amp;range=A",ROW())</t>
   </si>
 </sst>
 </file>

</xml_diff>